<commit_message>
Fix sign mismatches in transaction records and update cleaned bank data files
</commit_message>
<xml_diff>
--- a/Aug_5/Cleaned_bank_data.xlsx
+++ b/Aug_5/Cleaned_bank_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="170">
   <si>
     <t>transactionid</t>
   </si>
@@ -524,9 +524,6 @@
   </si>
   <si>
     <t>Merchant name typo?</t>
-  </si>
-  <si>
-    <t>Sign mismatch?</t>
   </si>
 </sst>
 </file>
@@ -1440,9 +1437,6 @@
       <c r="M14" t="s">
         <v>166</v>
       </c>
-      <c r="N14" t="s">
-        <v>170</v>
-      </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" t="s">
@@ -1483,9 +1477,6 @@
       </c>
       <c r="M15" t="s">
         <v>166</v>
-      </c>
-      <c r="N15" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:14">

</xml_diff>